<commit_message>
Ajout de la fonctionnalité X
</commit_message>
<xml_diff>
--- a/BILAN LOUMA PHASE1.xlsx
+++ b/BILAN LOUMA PHASE1.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="34">
   <si>
     <t>DR</t>
   </si>
@@ -99,13 +99,40 @@
   </si>
   <si>
     <t>TOT OM</t>
+  </si>
+  <si>
+    <t>M5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BILAN DES REALISATIONS SIM - JUILLET </t>
+  </si>
+  <si>
+    <t>SEM1</t>
+  </si>
+  <si>
+    <t>SEM2</t>
+  </si>
+  <si>
+    <t>SEM3</t>
+  </si>
+  <si>
+    <t>SEM4</t>
+  </si>
+  <si>
+    <t>TR</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                                                   </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -125,8 +152,43 @@
       <name val="Arial Black"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -142,6 +204,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF47D359"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -179,22 +259,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -203,9 +284,28 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Pourcentage" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -483,32 +583,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:I23"/>
+  <dimension ref="B1:T23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="2:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="2" t="s">
+    <row r="1" spans="2:20" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-    </row>
-    <row r="2" spans="2:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+    </row>
+    <row r="2" spans="2:20" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+    </row>
+    <row r="3" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -525,198 +627,305 @@
         <v>4</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B4" s="4" t="s">
+    <row r="4" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="2">
         <v>0</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="2">
         <v>1461</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="2">
         <v>1654</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="2">
         <v>1272</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="2">
+        <v>1402</v>
+      </c>
+      <c r="H4" s="2">
         <v>4387</v>
       </c>
-      <c r="H4" s="4">
+      <c r="I4" s="2">
         <v>2880</v>
       </c>
-      <c r="I4" s="5">
+      <c r="J4" s="3">
         <v>1.52</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B5" s="4" t="s">
+    <row r="5" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="2">
         <v>1017</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="2">
         <v>1529</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="2">
         <v>1736</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="2">
         <v>1009</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="2"/>
+      <c r="H5" s="2">
         <v>5291</v>
       </c>
-      <c r="H5" s="4">
+      <c r="I5" s="2">
         <v>3800</v>
       </c>
-      <c r="I5" s="5">
+      <c r="J5" s="3">
         <v>1.39</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B6" s="4" t="s">
+    <row r="6" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="2">
         <v>1026</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="2">
         <v>1421</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="2">
         <v>1533</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="2">
         <v>1056</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="2"/>
+      <c r="H6" s="2">
         <v>5036</v>
       </c>
-      <c r="H6" s="4">
+      <c r="I6" s="2">
         <v>3800</v>
       </c>
-      <c r="I6" s="5">
+      <c r="J6" s="3">
         <v>1.32</v>
       </c>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B7" s="4" t="s">
+      <c r="S6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="2">
         <v>513</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="2">
         <v>1166</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="2">
         <v>1286</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="2">
         <v>995</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="2"/>
+      <c r="H7" s="2">
         <v>3960</v>
       </c>
-      <c r="H7" s="4">
+      <c r="I7" s="2">
         <v>3800</v>
       </c>
-      <c r="I7" s="5">
+      <c r="J7" s="3">
         <v>1.04</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B8" s="4" t="s">
+    <row r="8" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="2">
         <v>595</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="2">
         <v>1182</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="2">
         <v>1503</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="2">
         <v>1054</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="2"/>
+      <c r="H8" s="2">
         <v>4334</v>
       </c>
-      <c r="H8" s="4">
+      <c r="I8" s="2">
         <v>3800</v>
       </c>
-      <c r="I8" s="5">
+      <c r="J8" s="3">
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B9" s="4" t="s">
+    <row r="9" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="2">
         <v>527</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="2">
         <v>1057</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="2">
         <v>1051</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="2">
         <v>731</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="2"/>
+      <c r="H9" s="2">
         <v>3366</v>
       </c>
-      <c r="H9" s="4">
+      <c r="I9" s="2">
         <v>3800</v>
       </c>
-      <c r="I9" s="5">
+      <c r="J9" s="3">
         <v>0.89</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B10" s="4" t="s">
+    <row r="10" spans="2:20" ht="21" x14ac:dyDescent="0.5">
+      <c r="B10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="2">
         <v>3678</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="2">
         <v>7816</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="2">
         <v>8763</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="2">
         <v>6117</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="2"/>
+      <c r="H10" s="2">
         <v>26374</v>
       </c>
-      <c r="H10" s="4">
+      <c r="I10" s="2">
         <v>21880</v>
       </c>
-      <c r="I10" s="5">
+      <c r="J10" s="3">
         <v>1.21</v>
       </c>
-    </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="M10" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N10" s="9"/>
+      <c r="O10" s="9"/>
+      <c r="P10" s="9"/>
+      <c r="Q10" s="9"/>
+      <c r="R10" s="9"/>
+      <c r="S10" s="9"/>
+      <c r="T10" s="9"/>
+    </row>
+    <row r="11" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="M11" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="O11" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="P11" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q11" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="R11" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="S11" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="T11" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="M12" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="N12" s="8">
+        <v>569</v>
+      </c>
+      <c r="O12" s="8">
+        <v>299</v>
+      </c>
+      <c r="P12" s="8">
+        <v>301</v>
+      </c>
+      <c r="Q12" s="8">
+        <v>233</v>
+      </c>
+      <c r="R12" s="8">
+        <f t="shared" ref="R12:R18" si="0">SUM(N12:Q12)</f>
+        <v>1402</v>
+      </c>
+      <c r="S12" s="8">
+        <v>960</v>
+      </c>
+      <c r="T12" s="11">
+        <f>R12/S12</f>
+        <v>1.4604166666666667</v>
+      </c>
+    </row>
+    <row r="13" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="M13" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="N13" s="8">
+        <v>230</v>
+      </c>
+      <c r="O13" s="8">
+        <v>225</v>
+      </c>
+      <c r="P13" s="8">
+        <v>240</v>
+      </c>
+      <c r="Q13" s="8">
+        <v>261</v>
+      </c>
+      <c r="R13" s="8">
+        <f t="shared" si="0"/>
+        <v>956</v>
+      </c>
+      <c r="S13" s="8">
+        <v>960</v>
+      </c>
+      <c r="T13" s="11">
+        <f>R13/S13</f>
+        <v>0.99583333333333335</v>
+      </c>
+    </row>
+    <row r="14" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B14" s="6" t="s">
         <v>23</v>
       </c>
@@ -727,8 +936,35 @@
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
-    </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="J14" s="6"/>
+      <c r="M14" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N14" s="8">
+        <v>356</v>
+      </c>
+      <c r="O14" s="8">
+        <v>275</v>
+      </c>
+      <c r="P14" s="8">
+        <v>318</v>
+      </c>
+      <c r="Q14" s="8">
+        <v>236</v>
+      </c>
+      <c r="R14" s="8">
+        <f t="shared" si="0"/>
+        <v>1185</v>
+      </c>
+      <c r="S14" s="8">
+        <v>960</v>
+      </c>
+      <c r="T14" s="11">
+        <f>R14/S14</f>
+        <v>1.234375</v>
+      </c>
+    </row>
+    <row r="15" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -737,8 +973,35 @@
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
       <c r="I15" s="7"/>
-    </row>
-    <row r="16" spans="2:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J15" s="7"/>
+      <c r="M15" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="N15" s="8">
+        <v>182</v>
+      </c>
+      <c r="O15" s="8">
+        <v>296</v>
+      </c>
+      <c r="P15" s="8">
+        <v>215</v>
+      </c>
+      <c r="Q15" s="8">
+        <v>248</v>
+      </c>
+      <c r="R15" s="8">
+        <f t="shared" si="0"/>
+        <v>941</v>
+      </c>
+      <c r="S15" s="8">
+        <v>960</v>
+      </c>
+      <c r="T15" s="12">
+        <f>+R15/S15</f>
+        <v>0.98020833333333335</v>
+      </c>
+    </row>
+    <row r="16" spans="2:20" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="1" t="s">
         <v>0</v>
       </c>
@@ -754,202 +1017,290 @@
       <c r="F16" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="G16" s="1"/>
+      <c r="H16" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="I16" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="J16" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B17" s="4" t="s">
+      <c r="M16" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="N16" s="8">
+        <v>287</v>
+      </c>
+      <c r="O16" s="8">
+        <v>313</v>
+      </c>
+      <c r="P16" s="8">
+        <v>304</v>
+      </c>
+      <c r="Q16" s="8">
+        <v>257</v>
+      </c>
+      <c r="R16" s="8">
+        <f t="shared" si="0"/>
+        <v>1161</v>
+      </c>
+      <c r="S16" s="8">
+        <v>960</v>
+      </c>
+      <c r="T16" s="11">
+        <f>+R16/S16</f>
+        <v>1.2093750000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="2">
         <v>0</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="2">
         <v>1099</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="2">
         <v>200</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="2">
         <v>86</v>
       </c>
-      <c r="G17" s="4">
+      <c r="G17" s="2"/>
+      <c r="H17" s="2">
         <v>1385</v>
       </c>
-      <c r="H17" s="4">
+      <c r="I17" s="2">
         <v>1440</v>
       </c>
-      <c r="I17" s="5" t="s">
+      <c r="J17" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B18" s="4" t="s">
+      <c r="M17" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="N17" s="8">
+        <v>238</v>
+      </c>
+      <c r="O17" s="8">
+        <v>255</v>
+      </c>
+      <c r="P17" s="8">
+        <v>209</v>
+      </c>
+      <c r="Q17" s="8">
+        <v>257</v>
+      </c>
+      <c r="R17" s="8">
+        <f t="shared" si="0"/>
+        <v>959</v>
+      </c>
+      <c r="S17" s="8">
+        <v>960</v>
+      </c>
+      <c r="T17" s="11">
+        <f>+R17/S17</f>
+        <v>0.99895833333333328</v>
+      </c>
+    </row>
+    <row r="18" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B18" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="4">
+      <c r="C18" s="2">
         <v>473</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="2">
         <v>753</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="2">
         <v>349</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="2">
         <v>185</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18" s="2"/>
+      <c r="H18" s="2">
         <v>1760</v>
       </c>
-      <c r="H18" s="4">
+      <c r="I18" s="2">
         <v>1920</v>
       </c>
-      <c r="I18" s="5" t="s">
+      <c r="J18" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B19" s="4" t="s">
+      <c r="M18" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="N18" s="10">
+        <v>1862</v>
+      </c>
+      <c r="O18" s="10">
+        <v>1663</v>
+      </c>
+      <c r="P18" s="10">
+        <v>1587</v>
+      </c>
+      <c r="Q18" s="8">
+        <v>1492</v>
+      </c>
+      <c r="R18" s="8">
+        <f t="shared" si="0"/>
+        <v>6604</v>
+      </c>
+      <c r="S18" s="8">
+        <f>SUM(S12:S17)</f>
+        <v>5760</v>
+      </c>
+      <c r="T18" s="13">
+        <f>+R18/S18</f>
+        <v>1.1465277777777778</v>
+      </c>
+    </row>
+    <row r="19" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B19" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="2">
         <v>526</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="2">
         <v>308</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="2">
         <v>220</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="2">
         <v>127</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19" s="2"/>
+      <c r="H19" s="2">
         <v>1181</v>
       </c>
-      <c r="H19" s="4">
+      <c r="I19" s="2">
         <v>1920</v>
       </c>
-      <c r="I19" s="5" t="s">
+      <c r="J19" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B20" s="4" t="s">
+    <row r="20" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B20" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C20" s="2">
         <v>630</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="2">
         <v>556</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="2">
         <v>131</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="2">
         <v>123</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G20" s="2"/>
+      <c r="H20" s="2">
         <v>1440</v>
       </c>
-      <c r="H20" s="4">
+      <c r="I20" s="2">
         <v>1920</v>
       </c>
-      <c r="I20" s="5" t="s">
+      <c r="J20" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B21" s="4" t="s">
+    <row r="21" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B21" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="2">
         <v>557</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="2">
         <v>180</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="2">
         <v>10</v>
       </c>
-      <c r="F21" s="4">
+      <c r="F21" s="2">
         <v>10</v>
       </c>
-      <c r="G21" s="4">
+      <c r="G21" s="2"/>
+      <c r="H21" s="2">
         <v>757</v>
       </c>
-      <c r="H21" s="4">
+      <c r="I21" s="2">
         <v>1920</v>
       </c>
-      <c r="I21" s="5" t="s">
+      <c r="J21" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B22" s="4" t="s">
+    <row r="22" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B22" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="2">
         <v>283</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="2">
         <v>77</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22" s="2">
         <v>3</v>
       </c>
-      <c r="F22" s="4">
+      <c r="F22" s="2">
         <v>3</v>
       </c>
-      <c r="G22" s="4">
+      <c r="G22" s="2"/>
+      <c r="H22" s="2">
         <v>366</v>
       </c>
-      <c r="H22" s="4">
+      <c r="I22" s="2">
         <v>1920</v>
       </c>
-      <c r="I22" s="5" t="s">
+      <c r="J22" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B23" s="4" t="s">
+    <row r="23" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="B23" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="4">
+      <c r="C23" s="2">
         <v>2469</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="2">
         <v>2973</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23" s="2">
         <v>913</v>
       </c>
-      <c r="F23" s="4">
+      <c r="F23" s="2">
         <v>534</v>
       </c>
-      <c r="G23" s="4">
+      <c r="G23" s="2"/>
+      <c r="H23" s="2">
         <v>6889</v>
       </c>
-      <c r="H23" s="4">
+      <c r="I23" s="2">
         <v>11040</v>
       </c>
-      <c r="I23" s="5" t="s">
+      <c r="J23" s="3" t="s">
         <v>22</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B1:I2"/>
-    <mergeCell ref="B14:I15"/>
+  <mergeCells count="3">
+    <mergeCell ref="B1:J2"/>
+    <mergeCell ref="B14:J15"/>
+    <mergeCell ref="M10:T10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -982,6 +1333,10 @@
               <xm:f>' BILAN LOUMA PHASE1 SIM&amp;OM'!F3:F3</xm:f>
               <xm:sqref>F3</xm:sqref>
             </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>' BILAN LOUMA PHASE1 SIM&amp;OM'!G3:G3</xm:f>
+              <xm:sqref>G3</xm:sqref>
+            </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
       </x14:sparklineGroups>

</xml_diff>